<commit_message>
Integra lector beta de facturas y mejoras de modulos
</commit_message>
<xml_diff>
--- a/utils/004 LUZ componentes regulados.xlsx
+++ b/utils/004 LUZ componentes regulados.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jovid\Documents\015 JOSE\070 ENERGIA\002 HERRAMIENTAS EXCEL\FUNCIONALES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45162D90-4A9D-430A-A10A-870B6C15DDA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4FCAD92-29B7-434A-A3DC-4E963105471C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{08F9EB0C-B30B-42B1-8987-81224755E03F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{08F9EB0C-B30B-42B1-8987-81224755E03F}"/>
   </bookViews>
   <sheets>
     <sheet name="PPCC" sheetId="1" r:id="rId1"/>
     <sheet name="OSOM" sheetId="2" r:id="rId2"/>
     <sheet name="PERDIDAS" sheetId="3" r:id="rId3"/>
     <sheet name="PYC_E" sheetId="4" r:id="rId4"/>
+    <sheet name="FBS" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="19">
   <si>
     <t>fecha_inicio</t>
   </si>
@@ -77,6 +78,15 @@
   <si>
     <t>osom</t>
   </si>
+  <si>
+    <t>fecha_ini</t>
+  </si>
+  <si>
+    <t>fecha_fin</t>
+  </si>
+  <si>
+    <t>importe_fbs</t>
+  </si>
 </sst>
 </file>
 
@@ -87,7 +97,7 @@
     <numFmt numFmtId="164" formatCode="0.000000"/>
     <numFmt numFmtId="165" formatCode="0.000000;\-0.000000;;@"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="9"/>
       <color theme="1"/>
@@ -176,6 +186,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -203,7 +219,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -231,6 +247,117 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -238,7 +365,7 @@
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -324,6 +451,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Millares" xfId="2" builtinId="3"/>
@@ -331,7 +485,169 @@
     <cellStyle name="Normal 2" xfId="3" xr:uid="{247834AE-F68A-4289-B3BE-CDD735F2F35F}"/>
     <cellStyle name="Normal 2 2" xfId="1" xr:uid="{41148CBB-D82C-43FF-AD12-143E4FA8120A}"/>
   </cellStyles>
-  <dxfs count="36">
+  <dxfs count="43">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right/>
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1222,69 +1538,80 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5502E831-9AD3-4C66-965A-DDE95429CB68}" name="T_PPCC" displayName="T_PPCC" ref="A1:I37" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34" headerRowCellStyle="Normal 2 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5502E831-9AD3-4C66-965A-DDE95429CB68}" name="T_PPCC" displayName="T_PPCC" ref="A1:I37" totalsRowShown="0" headerRowDxfId="42" dataDxfId="41" headerRowCellStyle="Normal 2 2">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{DFE4CBB5-BD00-426D-95D9-9CCCC0215AEF}" name="fecha_inicio" dataDxfId="33"/>
-    <tableColumn id="9" xr3:uid="{376051B5-C0AF-40DC-A15F-8C050C61AA1B}" name="fecha_final" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{021DD24A-8EDF-480B-87D6-753352E53592}" name="periodo" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{F4F697C2-1E95-4CF5-8222-09258654E24E}" name="2.0TD" dataDxfId="30" dataCellStyle="Normal 2 2"/>
-    <tableColumn id="4" xr3:uid="{D85305DC-1CC0-4298-8B8C-8DA40E54D211}" name="3.0TD" dataDxfId="29" dataCellStyle="Normal 2 2"/>
-    <tableColumn id="5" xr3:uid="{BD4ABDCF-C110-4A88-8DD8-1B955761E77F}" name="6.1TD" dataDxfId="28" dataCellStyle="Normal 2 2"/>
-    <tableColumn id="6" xr3:uid="{763694C5-6492-4D48-9576-D5DDC607C570}" name="6.2TD" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{6E4A1187-66FE-49B2-A79C-D5BF392D89D7}" name="6.3TD" dataDxfId="26"/>
-    <tableColumn id="8" xr3:uid="{7FEE70CD-8807-4EA8-893E-56229A131CA4}" name="6.4TD" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{DFE4CBB5-BD00-426D-95D9-9CCCC0215AEF}" name="fecha_inicio" dataDxfId="40"/>
+    <tableColumn id="9" xr3:uid="{376051B5-C0AF-40DC-A15F-8C050C61AA1B}" name="fecha_final" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{021DD24A-8EDF-480B-87D6-753352E53592}" name="periodo" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{F4F697C2-1E95-4CF5-8222-09258654E24E}" name="2.0TD" dataDxfId="37" dataCellStyle="Normal 2 2"/>
+    <tableColumn id="4" xr3:uid="{D85305DC-1CC0-4298-8B8C-8DA40E54D211}" name="3.0TD" dataDxfId="36" dataCellStyle="Normal 2 2"/>
+    <tableColumn id="5" xr3:uid="{BD4ABDCF-C110-4A88-8DD8-1B955761E77F}" name="6.1TD" dataDxfId="35" dataCellStyle="Normal 2 2"/>
+    <tableColumn id="6" xr3:uid="{763694C5-6492-4D48-9576-D5DDC607C570}" name="6.2TD" dataDxfId="34"/>
+    <tableColumn id="7" xr3:uid="{6E4A1187-66FE-49B2-A79C-D5BF392D89D7}" name="6.3TD" dataDxfId="33"/>
+    <tableColumn id="8" xr3:uid="{7FEE70CD-8807-4EA8-893E-56229A131CA4}" name="6.4TD" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{BDACDBEB-93E8-4337-BD28-6A50CA766471}" name="Tabla5" displayName="Tabla5" ref="A1:C7" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{BDACDBEB-93E8-4337-BD28-6A50CA766471}" name="Tabla5" displayName="Tabla5" ref="A1:C7" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{FFBAFEEB-7A62-4B5F-A756-D0EB7A8994E9}" name="fecha_inicio" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{76D4B312-18A1-4BEE-AD0B-47A2B16E4851}" name="fecha_final" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{2263249A-644D-4447-A7E3-E21C100168FD}" name="osom" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{FFBAFEEB-7A62-4B5F-A756-D0EB7A8994E9}" name="fecha_inicio" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{76D4B312-18A1-4BEE-AD0B-47A2B16E4851}" name="fecha_final" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{2263249A-644D-4447-A7E3-E21C100168FD}" name="osom" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{348E55D9-8A75-4585-9116-4ED36539FFF5}" name="T_PERDIDAS_TD_2" displayName="T_PERDIDAS_TD_2" ref="A1:G7" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{348E55D9-8A75-4585-9116-4ED36539FFF5}" name="T_PERDIDAS_TD_2" displayName="T_PERDIDAS_TD_2" ref="A1:G7" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{4B690220-9D4A-4F57-9F76-9A63DE61F284}" name="periodo" dataDxfId="17" dataCellStyle="Normal 2 2"/>
-    <tableColumn id="2" xr3:uid="{E7E69530-AA96-4398-B6FB-56B66F35C588}" name="2.0TD" dataDxfId="16" dataCellStyle="Millares"/>
-    <tableColumn id="3" xr3:uid="{DF8764BC-FABC-4EDB-9650-9DCB1DEADE29}" name="3.0TD" dataDxfId="15" dataCellStyle="Millares"/>
-    <tableColumn id="4" xr3:uid="{DFD26EFB-F437-43E2-BBC9-DE6A703E4C6F}" name="6.1TD" dataDxfId="14" dataCellStyle="Millares"/>
-    <tableColumn id="5" xr3:uid="{3F42E191-F3C1-4744-9929-6D95319544BE}" name="6.2TD" dataDxfId="13" dataCellStyle="Millares"/>
-    <tableColumn id="6" xr3:uid="{92EE04D1-24D6-4B54-8C7E-30531C949C1A}" name="6.3TD" dataDxfId="12" dataCellStyle="Millares"/>
-    <tableColumn id="7" xr3:uid="{312106D7-C4A3-46D7-9B5C-69C5274C0C26}" name="6.4TD" dataDxfId="11" dataCellStyle="Millares"/>
+    <tableColumn id="1" xr3:uid="{4B690220-9D4A-4F57-9F76-9A63DE61F284}" name="periodo" dataDxfId="24" dataCellStyle="Normal 2 2"/>
+    <tableColumn id="2" xr3:uid="{E7E69530-AA96-4398-B6FB-56B66F35C588}" name="2.0TD" dataDxfId="23" dataCellStyle="Millares"/>
+    <tableColumn id="3" xr3:uid="{DF8764BC-FABC-4EDB-9650-9DCB1DEADE29}" name="3.0TD" dataDxfId="22" dataCellStyle="Millares"/>
+    <tableColumn id="4" xr3:uid="{DFD26EFB-F437-43E2-BBC9-DE6A703E4C6F}" name="6.1TD" dataDxfId="21" dataCellStyle="Millares"/>
+    <tableColumn id="5" xr3:uid="{3F42E191-F3C1-4744-9929-6D95319544BE}" name="6.2TD" dataDxfId="20" dataCellStyle="Millares"/>
+    <tableColumn id="6" xr3:uid="{92EE04D1-24D6-4B54-8C7E-30531C949C1A}" name="6.3TD" dataDxfId="19" dataCellStyle="Millares"/>
+    <tableColumn id="7" xr3:uid="{312106D7-C4A3-46D7-9B5C-69C5274C0C26}" name="6.4TD" dataDxfId="18" dataCellStyle="Millares"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium10" showFirstColumn="1" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{9798FD41-4591-4BA7-B0ED-553D9DA39D85}" name="T_PYC_E" displayName="T_PYC_E" ref="A1:I49" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9" headerRowCellStyle="Normal 2 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{9798FD41-4591-4BA7-B0ED-553D9DA39D85}" name="T_PYC_E" displayName="T_PYC_E" ref="A1:I49" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal 2 2">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{E46415C2-253E-45C4-8AF5-C675D02C367E}" name="fecha_inicio" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{E226E94B-3B9F-49D3-9026-87C2F9D7966F}" name="fecha_final" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{E66DD275-8B6E-42F1-BE8F-ED30197B80E1}" name="periodo" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{83C85B02-CD55-49BA-922A-75D8A0E72374}" name="2.0TD" dataDxfId="5" dataCellStyle="Normal 2 2"/>
-    <tableColumn id="4" xr3:uid="{AFB4561F-09B1-443E-B91B-E38DE7F466E9}" name="3.0TD" dataDxfId="4" dataCellStyle="Normal 2 2"/>
-    <tableColumn id="5" xr3:uid="{7F05503C-D77F-4C82-BFCE-FEEDE50EA53A}" name="6.1TD" dataDxfId="3" dataCellStyle="Normal 2 2"/>
-    <tableColumn id="6" xr3:uid="{1501CF01-7819-440F-9560-C6B0EDDC1D49}" name="6.2TD" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{00864210-9A71-4F0D-9C22-27B3912DB112}" name="6.3TD" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{57115F02-05F6-4484-935A-4B21F4D9CA86}" name="6.4TD" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{E46415C2-253E-45C4-8AF5-C675D02C367E}" name="fecha_inicio" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{E226E94B-3B9F-49D3-9026-87C2F9D7966F}" name="fecha_final" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{E66DD275-8B6E-42F1-BE8F-ED30197B80E1}" name="periodo" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{83C85B02-CD55-49BA-922A-75D8A0E72374}" name="2.0TD" dataDxfId="12" dataCellStyle="Normal 2 2"/>
+    <tableColumn id="4" xr3:uid="{AFB4561F-09B1-443E-B91B-E38DE7F466E9}" name="3.0TD" dataDxfId="11" dataCellStyle="Normal 2 2"/>
+    <tableColumn id="5" xr3:uid="{7F05503C-D77F-4C82-BFCE-FEEDE50EA53A}" name="6.1TD" dataDxfId="10" dataCellStyle="Normal 2 2"/>
+    <tableColumn id="6" xr3:uid="{1501CF01-7819-440F-9560-C6B0EDDC1D49}" name="6.2TD" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{00864210-9A71-4F0D-9C22-27B3912DB112}" name="6.3TD" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{57115F02-05F6-4484-935A-4B21F4D9CA86}" name="6.4TD" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B53E67BF-C00A-4A9A-B648-258F63077BFF}" name="Tabla2" displayName="Tabla2" ref="A1:C4" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="5" tableBorderDxfId="6" totalsRowBorderDxfId="4">
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{EB541510-222B-4ECB-B01F-17B2AA13ECA0}" name="fecha_ini" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{52743116-6831-476C-915E-6D5015546968}" name="fecha_fin" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{A600AEE7-F549-4D99-B449-EBD06EACB609}" name="importe_fbs" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1322,7 +1649,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1428,7 +1755,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1570,7 +1897,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4278,4 +4605,64 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48A2ED1A-E990-4882-B32A-95546B42E6DF}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="32" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="34" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="30">
+        <v>45292</v>
+      </c>
+      <c r="B2" s="29">
+        <v>45657</v>
+      </c>
+      <c r="C2" s="31">
+        <v>6.2820000000000003E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="30">
+        <v>45658</v>
+      </c>
+      <c r="B3" s="29">
+        <v>46022</v>
+      </c>
+      <c r="C3" s="31">
+        <v>1.2742E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="35">
+        <v>46023</v>
+      </c>
+      <c r="B4" s="36">
+        <v>46387</v>
+      </c>
+      <c r="C4" s="37">
+        <v>1.9120999999999999E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
añadido verificacion de factura con curva de carga
</commit_message>
<xml_diff>
--- a/utils/004 LUZ componentes regulados.xlsx
+++ b/utils/004 LUZ componentes regulados.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jovid\Documents\015 JOSE\070 ENERGIA\002 HERRAMIENTAS EXCEL\FUNCIONALES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4FCAD92-29B7-434A-A3DC-4E963105471C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985A87DC-DD7D-4DD1-BA67-55DD1648ED7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{08F9EB0C-B30B-42B1-8987-81224755E03F}"/>
   </bookViews>
@@ -486,168 +486,6 @@
     <cellStyle name="Normal 2 2" xfId="1" xr:uid="{41148CBB-D82C-43FF-AD12-143E4FA8120A}"/>
   </cellStyles>
   <dxfs count="43">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FFCCCCCC"/>
-        </left>
-        <right style="medium">
-          <color rgb="FFCCCCCC"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color rgb="FFCCCCCC"/>
-        </left>
-        <right/>
-        <top style="medium">
-          <color rgb="FFCCCCCC"/>
-        </top>
-        <bottom style="medium">
-          <color rgb="FFCCCCCC"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color rgb="FFCCCCCC"/>
-        </left>
-        <right style="medium">
-          <color rgb="FFCCCCCC"/>
-        </right>
-        <top style="medium">
-          <color rgb="FFCCCCCC"/>
-        </top>
-        <bottom style="medium">
-          <color rgb="FFCCCCCC"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="medium">
-          <color rgb="FFCCCCCC"/>
-        </right>
-        <top style="medium">
-          <color rgb="FFCCCCCC"/>
-        </top>
-        <bottom style="medium">
-          <color rgb="FFCCCCCC"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="medium">
-          <color rgb="FFCCCCCC"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="medium">
-          <color rgb="FFCCCCCC"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="medium">
-          <color rgb="FFCCCCCC"/>
-        </left>
-        <right style="medium">
-          <color rgb="FFCCCCCC"/>
-        </right>
-        <top style="medium">
-          <color rgb="FFCCCCCC"/>
-        </top>
-        <bottom style="medium">
-          <color rgb="FFCCCCCC"/>
-        </bottom>
-      </border>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1524,6 +1362,168 @@
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right/>
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFCCCCCC"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1538,71 +1538,71 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5502E831-9AD3-4C66-965A-DDE95429CB68}" name="T_PPCC" displayName="T_PPCC" ref="A1:I37" totalsRowShown="0" headerRowDxfId="42" dataDxfId="41" headerRowCellStyle="Normal 2 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5502E831-9AD3-4C66-965A-DDE95429CB68}" name="T_PPCC" displayName="T_PPCC" ref="A1:I37" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34" headerRowCellStyle="Normal 2 2">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{DFE4CBB5-BD00-426D-95D9-9CCCC0215AEF}" name="fecha_inicio" dataDxfId="40"/>
-    <tableColumn id="9" xr3:uid="{376051B5-C0AF-40DC-A15F-8C050C61AA1B}" name="fecha_final" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{021DD24A-8EDF-480B-87D6-753352E53592}" name="periodo" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{F4F697C2-1E95-4CF5-8222-09258654E24E}" name="2.0TD" dataDxfId="37" dataCellStyle="Normal 2 2"/>
-    <tableColumn id="4" xr3:uid="{D85305DC-1CC0-4298-8B8C-8DA40E54D211}" name="3.0TD" dataDxfId="36" dataCellStyle="Normal 2 2"/>
-    <tableColumn id="5" xr3:uid="{BD4ABDCF-C110-4A88-8DD8-1B955761E77F}" name="6.1TD" dataDxfId="35" dataCellStyle="Normal 2 2"/>
-    <tableColumn id="6" xr3:uid="{763694C5-6492-4D48-9576-D5DDC607C570}" name="6.2TD" dataDxfId="34"/>
-    <tableColumn id="7" xr3:uid="{6E4A1187-66FE-49B2-A79C-D5BF392D89D7}" name="6.3TD" dataDxfId="33"/>
-    <tableColumn id="8" xr3:uid="{7FEE70CD-8807-4EA8-893E-56229A131CA4}" name="6.4TD" dataDxfId="32"/>
+    <tableColumn id="1" xr3:uid="{DFE4CBB5-BD00-426D-95D9-9CCCC0215AEF}" name="fecha_inicio" dataDxfId="33"/>
+    <tableColumn id="9" xr3:uid="{376051B5-C0AF-40DC-A15F-8C050C61AA1B}" name="fecha_final" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{021DD24A-8EDF-480B-87D6-753352E53592}" name="periodo" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{F4F697C2-1E95-4CF5-8222-09258654E24E}" name="2.0TD" dataDxfId="30" dataCellStyle="Normal 2 2"/>
+    <tableColumn id="4" xr3:uid="{D85305DC-1CC0-4298-8B8C-8DA40E54D211}" name="3.0TD" dataDxfId="29" dataCellStyle="Normal 2 2"/>
+    <tableColumn id="5" xr3:uid="{BD4ABDCF-C110-4A88-8DD8-1B955761E77F}" name="6.1TD" dataDxfId="28" dataCellStyle="Normal 2 2"/>
+    <tableColumn id="6" xr3:uid="{763694C5-6492-4D48-9576-D5DDC607C570}" name="6.2TD" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{6E4A1187-66FE-49B2-A79C-D5BF392D89D7}" name="6.3TD" dataDxfId="26"/>
+    <tableColumn id="8" xr3:uid="{7FEE70CD-8807-4EA8-893E-56229A131CA4}" name="6.4TD" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{BDACDBEB-93E8-4337-BD28-6A50CA766471}" name="Tabla5" displayName="Tabla5" ref="A1:C7" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{BDACDBEB-93E8-4337-BD28-6A50CA766471}" name="Tabla5" displayName="Tabla5" ref="A1:C7" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{FFBAFEEB-7A62-4B5F-A756-D0EB7A8994E9}" name="fecha_inicio" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{76D4B312-18A1-4BEE-AD0B-47A2B16E4851}" name="fecha_final" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{2263249A-644D-4447-A7E3-E21C100168FD}" name="osom" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{FFBAFEEB-7A62-4B5F-A756-D0EB7A8994E9}" name="fecha_inicio" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{76D4B312-18A1-4BEE-AD0B-47A2B16E4851}" name="fecha_final" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{2263249A-644D-4447-A7E3-E21C100168FD}" name="osom" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{348E55D9-8A75-4585-9116-4ED36539FFF5}" name="T_PERDIDAS_TD_2" displayName="T_PERDIDAS_TD_2" ref="A1:G7" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{348E55D9-8A75-4585-9116-4ED36539FFF5}" name="T_PERDIDAS_TD_2" displayName="T_PERDIDAS_TD_2" ref="A1:G7" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{4B690220-9D4A-4F57-9F76-9A63DE61F284}" name="periodo" dataDxfId="24" dataCellStyle="Normal 2 2"/>
-    <tableColumn id="2" xr3:uid="{E7E69530-AA96-4398-B6FB-56B66F35C588}" name="2.0TD" dataDxfId="23" dataCellStyle="Millares"/>
-    <tableColumn id="3" xr3:uid="{DF8764BC-FABC-4EDB-9650-9DCB1DEADE29}" name="3.0TD" dataDxfId="22" dataCellStyle="Millares"/>
-    <tableColumn id="4" xr3:uid="{DFD26EFB-F437-43E2-BBC9-DE6A703E4C6F}" name="6.1TD" dataDxfId="21" dataCellStyle="Millares"/>
-    <tableColumn id="5" xr3:uid="{3F42E191-F3C1-4744-9929-6D95319544BE}" name="6.2TD" dataDxfId="20" dataCellStyle="Millares"/>
-    <tableColumn id="6" xr3:uid="{92EE04D1-24D6-4B54-8C7E-30531C949C1A}" name="6.3TD" dataDxfId="19" dataCellStyle="Millares"/>
-    <tableColumn id="7" xr3:uid="{312106D7-C4A3-46D7-9B5C-69C5274C0C26}" name="6.4TD" dataDxfId="18" dataCellStyle="Millares"/>
+    <tableColumn id="1" xr3:uid="{4B690220-9D4A-4F57-9F76-9A63DE61F284}" name="periodo" dataDxfId="17" dataCellStyle="Normal 2 2"/>
+    <tableColumn id="2" xr3:uid="{E7E69530-AA96-4398-B6FB-56B66F35C588}" name="2.0TD" dataDxfId="16" dataCellStyle="Millares"/>
+    <tableColumn id="3" xr3:uid="{DF8764BC-FABC-4EDB-9650-9DCB1DEADE29}" name="3.0TD" dataDxfId="15" dataCellStyle="Millares"/>
+    <tableColumn id="4" xr3:uid="{DFD26EFB-F437-43E2-BBC9-DE6A703E4C6F}" name="6.1TD" dataDxfId="14" dataCellStyle="Millares"/>
+    <tableColumn id="5" xr3:uid="{3F42E191-F3C1-4744-9929-6D95319544BE}" name="6.2TD" dataDxfId="13" dataCellStyle="Millares"/>
+    <tableColumn id="6" xr3:uid="{92EE04D1-24D6-4B54-8C7E-30531C949C1A}" name="6.3TD" dataDxfId="12" dataCellStyle="Millares"/>
+    <tableColumn id="7" xr3:uid="{312106D7-C4A3-46D7-9B5C-69C5274C0C26}" name="6.4TD" dataDxfId="11" dataCellStyle="Millares"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium10" showFirstColumn="1" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{9798FD41-4591-4BA7-B0ED-553D9DA39D85}" name="T_PYC_E" displayName="T_PYC_E" ref="A1:I49" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16" headerRowCellStyle="Normal 2 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{9798FD41-4591-4BA7-B0ED-553D9DA39D85}" name="T_PYC_E" displayName="T_PYC_E" ref="A1:I49" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9" headerRowCellStyle="Normal 2 2">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{E46415C2-253E-45C4-8AF5-C675D02C367E}" name="fecha_inicio" dataDxfId="15"/>
-    <tableColumn id="9" xr3:uid="{E226E94B-3B9F-49D3-9026-87C2F9D7966F}" name="fecha_final" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{E66DD275-8B6E-42F1-BE8F-ED30197B80E1}" name="periodo" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{83C85B02-CD55-49BA-922A-75D8A0E72374}" name="2.0TD" dataDxfId="12" dataCellStyle="Normal 2 2"/>
-    <tableColumn id="4" xr3:uid="{AFB4561F-09B1-443E-B91B-E38DE7F466E9}" name="3.0TD" dataDxfId="11" dataCellStyle="Normal 2 2"/>
-    <tableColumn id="5" xr3:uid="{7F05503C-D77F-4C82-BFCE-FEEDE50EA53A}" name="6.1TD" dataDxfId="10" dataCellStyle="Normal 2 2"/>
-    <tableColumn id="6" xr3:uid="{1501CF01-7819-440F-9560-C6B0EDDC1D49}" name="6.2TD" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{00864210-9A71-4F0D-9C22-27B3912DB112}" name="6.3TD" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{57115F02-05F6-4484-935A-4B21F4D9CA86}" name="6.4TD" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{E46415C2-253E-45C4-8AF5-C675D02C367E}" name="fecha_inicio" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{E226E94B-3B9F-49D3-9026-87C2F9D7966F}" name="fecha_final" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{E66DD275-8B6E-42F1-BE8F-ED30197B80E1}" name="periodo" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{83C85B02-CD55-49BA-922A-75D8A0E72374}" name="2.0TD" dataDxfId="5" dataCellStyle="Normal 2 2"/>
+    <tableColumn id="4" xr3:uid="{AFB4561F-09B1-443E-B91B-E38DE7F466E9}" name="3.0TD" dataDxfId="4" dataCellStyle="Normal 2 2"/>
+    <tableColumn id="5" xr3:uid="{7F05503C-D77F-4C82-BFCE-FEEDE50EA53A}" name="6.1TD" dataDxfId="3" dataCellStyle="Normal 2 2"/>
+    <tableColumn id="6" xr3:uid="{1501CF01-7819-440F-9560-C6B0EDDC1D49}" name="6.2TD" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{00864210-9A71-4F0D-9C22-27B3912DB112}" name="6.3TD" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{57115F02-05F6-4484-935A-4B21F4D9CA86}" name="6.4TD" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B53E67BF-C00A-4A9A-B648-258F63077BFF}" name="Tabla2" displayName="Tabla2" ref="A1:C4" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="5" tableBorderDxfId="6" totalsRowBorderDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B53E67BF-C00A-4A9A-B648-258F63077BFF}" name="Tabla2" displayName="Tabla2" ref="A1:C5" totalsRowShown="0" headerRowDxfId="42" headerRowBorderDxfId="41" tableBorderDxfId="40" totalsRowBorderDxfId="39">
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{EB541510-222B-4ECB-B01F-17B2AA13ECA0}" name="fecha_ini" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{52743116-6831-476C-915E-6D5015546968}" name="fecha_fin" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{A600AEE7-F549-4D99-B449-EBD06EACB609}" name="importe_fbs" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{EB541510-222B-4ECB-B01F-17B2AA13ECA0}" name="fecha_ini" dataDxfId="38"/>
+    <tableColumn id="2" xr3:uid="{52743116-6831-476C-915E-6D5015546968}" name="fecha_fin" dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{A600AEE7-F549-4D99-B449-EBD06EACB609}" name="importe_fbs" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4609,7 +4609,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48A2ED1A-E990-4882-B32A-95546B42E6DF}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="13.5703125" customWidth="1"/>
@@ -4648,16 +4648,32 @@
         <v>1.2742E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="35">
         <v>46023</v>
       </c>
       <c r="B4" s="36">
-        <v>46387</v>
+        <v>46198</v>
       </c>
       <c r="C4" s="37">
         <v>1.9120999999999999E-2</v>
       </c>
+    </row>
+    <row r="5" spans="1:3" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="35">
+        <v>46199</v>
+      </c>
+      <c r="B5" s="36">
+        <v>46387</v>
+      </c>
+      <c r="C5" s="37">
+        <v>2.4688999999999999E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A6" s="35"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="37"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>